<commit_message>
Replace repository with manuscript code, data and results archive
</commit_message>
<xml_diff>
--- a/data/parallaxes_1.xlsx
+++ b/data/parallaxes_1.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11600"/>
+    <workbookView windowWidth="28800" windowHeight="12200"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="140">
   <si>
     <t>Jname</t>
   </si>
@@ -57,6 +57,18 @@
   </si>
   <si>
     <t>Binary</t>
+  </si>
+  <si>
+    <t>pmra</t>
+  </si>
+  <si>
+    <t>pmdec</t>
+  </si>
+  <si>
+    <t>gl</t>
+  </si>
+  <si>
+    <t>gb</t>
   </si>
   <si>
     <t>J0030+0451</t>
@@ -447,13 +459,19 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="22">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial Unicode MS"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
@@ -926,16 +944,13 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -944,123 +959,129 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1588,7 +1609,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J101"/>
+  <dimension ref="A1:N101"/>
   <sheetFormatPr defaultColWidth="9.23076923076923" defaultRowHeight="16.8"/>
   <cols>
     <col min="1" max="1" width="12.6923076923077" customWidth="1"/>
@@ -1598,7 +1619,7 @@
     <col min="7" max="9" width="12.6923076923077" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:14">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1629,10 +1650,22 @@
       <c r="J1" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="2" spans="1:10">
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B2">
         <v>3.03</v>
@@ -1644,10 +1677,10 @@
         <v>0.06</v>
       </c>
       <c r="E2" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F2" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G2">
         <v>0.005</v>
@@ -1659,12 +1692,12 @@
         <v>758</v>
       </c>
       <c r="J2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B3">
         <v>0.93</v>
@@ -1676,10 +1709,10 @@
         <v>0.07</v>
       </c>
       <c r="E3" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F3" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G3">
         <v>0.943</v>
@@ -1691,12 +1724,24 @@
         <v>3.65</v>
       </c>
       <c r="J3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K3">
+        <v>10.37</v>
+      </c>
+      <c r="L3">
+        <v>-11.13</v>
+      </c>
+      <c r="M3">
+        <v>110.42</v>
+      </c>
+      <c r="N3">
+        <v>-69.815</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B4">
         <v>0.102</v>
@@ -1708,10 +1753,10 @@
         <v>0.025</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F4" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G4">
         <v>1.118</v>
@@ -1723,12 +1768,24 @@
         <v>0.615</v>
       </c>
       <c r="J4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K4">
+        <v>12.39</v>
+      </c>
+      <c r="L4">
+        <v>-5.4</v>
+      </c>
+      <c r="M4" s="1">
+        <v>121.452</v>
+      </c>
+      <c r="N4" s="1">
+        <v>-5.567</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B5">
         <v>0.35</v>
@@ -1740,10 +1797,10 @@
         <v>0.06</v>
       </c>
       <c r="E5" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F5" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G5">
         <v>2.115</v>
@@ -1755,12 +1812,24 @@
         <v>0.351</v>
       </c>
       <c r="J5" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K5">
+        <v>10.47</v>
+      </c>
+      <c r="L5">
+        <v>-17.4</v>
+      </c>
+      <c r="M5">
+        <v>123.621</v>
+      </c>
+      <c r="N5">
+        <v>-11.576</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B6">
         <v>0.4</v>
@@ -1772,10 +1841,10 @@
         <v>0.04</v>
       </c>
       <c r="E6" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F6" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G6">
         <v>1.679</v>
@@ -1787,12 +1856,24 @@
         <v>0.447</v>
       </c>
       <c r="J6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K6">
+        <v>9.24</v>
+      </c>
+      <c r="L6">
+        <v>1.77</v>
+      </c>
+      <c r="M6">
+        <v>124.08</v>
+      </c>
+      <c r="N6">
+        <v>2.773</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B7">
         <v>4.2</v>
@@ -1804,10 +1885,10 @@
         <v>1.4</v>
       </c>
       <c r="E7" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F7" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G7">
         <v>0.808</v>
@@ -1819,12 +1900,24 @@
         <v>32.2</v>
       </c>
       <c r="J7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K7">
+        <v>75</v>
+      </c>
+      <c r="L7">
+        <v>-152.5</v>
+      </c>
+      <c r="M7">
+        <v>140.93</v>
+      </c>
+      <c r="N7">
+        <v>-76.815</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
       <c r="A8" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B8">
         <v>0.47</v>
@@ -1836,10 +1929,10 @@
         <v>0.03</v>
       </c>
       <c r="E8" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F8" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G8">
         <v>1.284</v>
@@ -1851,12 +1944,24 @@
         <v>0.156</v>
       </c>
       <c r="J8" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K8">
+        <v>-32.75</v>
+      </c>
+      <c r="L8">
+        <v>35.15</v>
+      </c>
+      <c r="M8">
+        <v>124.646</v>
+      </c>
+      <c r="N8">
+        <v>3.328</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B9">
         <v>0.37</v>
@@ -1868,10 +1973,10 @@
         <v>0.04</v>
       </c>
       <c r="E9" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F9" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G9">
         <v>0.272</v>
@@ -1883,12 +1988,24 @@
         <v>0.0403</v>
       </c>
       <c r="J9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K9">
+        <v>-19.11</v>
+      </c>
+      <c r="L9">
+        <v>-16.6</v>
+      </c>
+      <c r="M9">
+        <v>129.216</v>
+      </c>
+      <c r="N9">
+        <v>-4.044</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B10">
         <v>0.49</v>
@@ -1900,10 +2017,10 @@
         <v>0.09</v>
       </c>
       <c r="E10" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F10" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G10">
         <v>0.196</v>
@@ -1915,12 +2032,24 @@
         <v>1.21</v>
       </c>
       <c r="J10" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K10">
+        <v>-6.39</v>
+      </c>
+      <c r="L10">
+        <v>3.8</v>
+      </c>
+      <c r="M10">
+        <v>130.059</v>
+      </c>
+      <c r="N10">
+        <v>-2.723</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B11">
         <v>0.22</v>
@@ -1932,10 +2061,10 @@
         <v>0.08</v>
       </c>
       <c r="E11" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F11" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G11">
         <v>1.465</v>
@@ -1947,12 +2076,12 @@
         <v>5.33</v>
       </c>
       <c r="J11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10">
-      <c r="A12" s="1" t="s">
-        <v>26</v>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
+      <c r="A12" s="2" t="s">
+        <v>30</v>
       </c>
       <c r="B12">
         <v>0.44</v>
@@ -1964,10 +2093,10 @@
         <v>0.18</v>
       </c>
       <c r="E12" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F12" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G12">
         <v>0.833</v>
@@ -1979,12 +2108,12 @@
         <v>1.01</v>
       </c>
       <c r="J12" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10">
-      <c r="A13" s="1" t="s">
-        <v>27</v>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
+      <c r="A13" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="B13">
         <v>0.554</v>
@@ -1996,10 +2125,10 @@
         <v>0.024</v>
       </c>
       <c r="E13" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F13" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G13">
         <v>2.352</v>
@@ -2011,12 +2140,24 @@
         <v>0.0197</v>
       </c>
       <c r="J13" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K13">
+        <v>1.57</v>
+      </c>
+      <c r="L13">
+        <v>44.8</v>
+      </c>
+      <c r="M13">
+        <v>130.586</v>
+      </c>
+      <c r="N13">
+        <v>0.326</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
       <c r="A14" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B14">
         <v>1.05</v>
@@ -2028,10 +2169,10 @@
         <v>0.04</v>
       </c>
       <c r="E14" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F14" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G14">
         <v>3.032</v>
@@ -2043,12 +2184,24 @@
         <v>7.56</v>
       </c>
       <c r="J14" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K14">
+        <v>26.5</v>
+      </c>
+      <c r="L14">
+        <v>-30.77</v>
+      </c>
+      <c r="M14">
+        <v>152.18</v>
+      </c>
+      <c r="N14">
+        <v>-14.338</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14">
       <c r="A15" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B15">
         <v>0.595</v>
@@ -2060,10 +2213,10 @@
         <v>0.025</v>
       </c>
       <c r="E15" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F15" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G15">
         <v>0.715</v>
@@ -2075,12 +2228,24 @@
         <v>0.553</v>
       </c>
       <c r="J15" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K15">
+        <v>16.97</v>
+      </c>
+      <c r="L15">
+        <v>-10.37</v>
+      </c>
+      <c r="M15">
+        <v>144.995</v>
+      </c>
+      <c r="N15">
+        <v>-1.221</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14">
       <c r="A16" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B16">
         <v>0.409</v>
@@ -2092,10 +2257,10 @@
         <v>0.027</v>
       </c>
       <c r="E16" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F16" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G16">
         <v>0.269</v>
@@ -2107,12 +2272,24 @@
         <v>58</v>
       </c>
       <c r="J16" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K16">
+        <v>-3.66</v>
+      </c>
+      <c r="L16">
+        <v>-0.08</v>
+      </c>
+      <c r="M16">
+        <v>150.348</v>
+      </c>
+      <c r="N16">
+        <v>-8.038</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14">
       <c r="A17" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B17">
         <v>0.305</v>
@@ -2124,10 +2301,10 @@
         <v>0.077</v>
       </c>
       <c r="E17" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F17" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G17">
         <v>0.197</v>
@@ -2139,12 +2316,24 @@
         <v>0.655</v>
       </c>
       <c r="J17" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K17">
+        <v>13.88</v>
+      </c>
+      <c r="L17">
+        <v>-10.61</v>
+      </c>
+      <c r="M17">
+        <v>149.099</v>
+      </c>
+      <c r="N17">
+        <v>-0.522</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14">
       <c r="A18" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B18">
         <v>0.91</v>
@@ -2156,10 +2345,10 @@
         <v>0.16</v>
       </c>
       <c r="E18" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F18" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="G18">
         <v>0.156</v>
@@ -2171,12 +2360,24 @@
         <v>0.0564</v>
       </c>
       <c r="J18" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K18">
+        <v>9.3</v>
+      </c>
+      <c r="L18">
+        <v>8.3</v>
+      </c>
+      <c r="M18">
+        <v>148.19</v>
+      </c>
+      <c r="N18">
+        <v>0.811</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14">
       <c r="A19" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B19">
         <v>0.22</v>
@@ -2188,10 +2389,10 @@
         <v>0.06</v>
       </c>
       <c r="E19" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F19" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G19">
         <v>0.595</v>
@@ -2203,12 +2404,24 @@
         <v>0.169</v>
       </c>
       <c r="J19" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K19">
+        <v>12.4</v>
+      </c>
+      <c r="L19">
+        <v>22.74</v>
+      </c>
+      <c r="M19">
+        <v>144.025</v>
+      </c>
+      <c r="N19">
+        <v>7.046</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14">
       <c r="A20" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B20">
         <v>0.65</v>
@@ -2220,10 +2433,10 @@
         <v>0.6</v>
       </c>
       <c r="E20" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F20" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G20">
         <v>0.549</v>
@@ -2235,12 +2448,12 @@
         <v>0.151</v>
       </c>
       <c r="J20" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14">
       <c r="A21" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B21">
         <v>0.84</v>
@@ -2252,10 +2465,10 @@
         <v>0.05</v>
       </c>
       <c r="E21" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F21" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G21">
         <v>0.341</v>
@@ -2267,12 +2480,24 @@
         <v>0.228</v>
       </c>
       <c r="J21" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K21">
+        <v>53.34</v>
+      </c>
+      <c r="L21">
+        <v>-17.56</v>
+      </c>
+      <c r="M21">
+        <v>152.617</v>
+      </c>
+      <c r="N21">
+        <v>7.547</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14">
       <c r="A22" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B22">
         <v>0.53</v>
@@ -2284,10 +2509,10 @@
         <v>0.06</v>
       </c>
       <c r="E22" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F22" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="G22">
         <v>0.033</v>
@@ -2299,12 +2524,12 @@
         <v>0.000126</v>
       </c>
       <c r="J22" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14">
       <c r="A23" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B23">
         <v>0.72</v>
@@ -2316,10 +2541,10 @@
         <v>0.09</v>
       </c>
       <c r="E23" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F23" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G23">
         <v>0.143</v>
@@ -2331,12 +2556,24 @@
         <v>0.0618</v>
       </c>
       <c r="J23" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K23">
+        <v>-23.57</v>
+      </c>
+      <c r="L23">
+        <v>52.87</v>
+      </c>
+      <c r="M23">
+        <v>179.719</v>
+      </c>
+      <c r="N23">
+        <v>-1.686</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14">
       <c r="A24" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B24">
         <v>0.48</v>
@@ -2348,10 +2585,10 @@
         <v>0.04</v>
       </c>
       <c r="E24" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F24" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G24">
         <v>0.396</v>
@@ -2363,12 +2600,24 @@
         <v>0.482</v>
       </c>
       <c r="J24" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K24">
+        <v>-7.36</v>
+      </c>
+      <c r="L24">
+        <v>-15.24</v>
+      </c>
+      <c r="M24">
+        <v>212.199</v>
+      </c>
+      <c r="N24">
+        <v>-13.481</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14">
       <c r="A25" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B25">
         <v>0.282</v>
@@ -2380,10 +2629,10 @@
         <v>0.031</v>
       </c>
       <c r="E25" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F25" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G25">
         <v>0.335</v>
@@ -2395,12 +2644,24 @@
         <v>0.00893</v>
       </c>
       <c r="J25" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K25">
+        <v>-0.024</v>
+      </c>
+      <c r="L25">
+        <v>-1.25</v>
+      </c>
+      <c r="M25">
+        <v>188.795</v>
+      </c>
+      <c r="N25">
+        <v>2.394</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14">
       <c r="A26" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B26">
         <v>0.33</v>
@@ -2412,10 +2673,10 @@
         <v>0.05</v>
       </c>
       <c r="E26" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F26" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G26">
         <v>0.477</v>
@@ -2427,12 +2688,24 @@
         <v>0.378</v>
       </c>
       <c r="J26" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K26">
+        <v>3.56</v>
+      </c>
+      <c r="L26">
+        <v>-4.68</v>
+      </c>
+      <c r="M26">
+        <v>188.817</v>
+      </c>
+      <c r="N26">
+        <v>6.223</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14">
       <c r="A27" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B27">
         <v>3</v>
@@ -2444,10 +2717,10 @@
         <v>0.4</v>
       </c>
       <c r="E27" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F27" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G27">
         <v>1.244</v>
@@ -2459,12 +2732,24 @@
         <v>0.274</v>
       </c>
       <c r="J27" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K27">
+        <v>-46.3</v>
+      </c>
+      <c r="L27">
+        <v>21.3</v>
+      </c>
+      <c r="M27">
+        <v>236.952</v>
+      </c>
+      <c r="N27">
+        <v>-16.758</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14">
       <c r="A28" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B28">
         <v>4</v>
@@ -2476,10 +2761,10 @@
         <v>1.3</v>
       </c>
       <c r="E28" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F28" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="G28">
         <v>0.237</v>
@@ -2491,12 +2776,24 @@
         <v>0.00342</v>
       </c>
       <c r="J28" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K28">
+        <v>138</v>
+      </c>
+      <c r="L28">
+        <v>97</v>
+      </c>
+      <c r="M28">
+        <v>195.134</v>
+      </c>
+      <c r="N28">
+        <v>4.266</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14">
       <c r="A29" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B29">
         <v>1.4</v>
@@ -2508,10 +2805,10 @@
         <v>0.4</v>
       </c>
       <c r="E29" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F29" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="G29">
         <v>0.009</v>
@@ -2523,12 +2820,12 @@
         <v>2850</v>
       </c>
       <c r="J29" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14">
       <c r="A30" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B30">
         <v>3.47</v>
@@ -2540,10 +2837,10 @@
         <v>0.36</v>
       </c>
       <c r="E30" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F30" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G30">
         <v>0.385</v>
@@ -2555,12 +2852,24 @@
         <v>0.0111</v>
       </c>
       <c r="J30" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K30">
+        <v>44.1</v>
+      </c>
+      <c r="L30">
+        <v>-2.4</v>
+      </c>
+      <c r="M30">
+        <v>201.108</v>
+      </c>
+      <c r="N30">
+        <v>8.258</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14">
       <c r="A31" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B31">
         <v>2.77</v>
@@ -2572,10 +2881,10 @@
         <v>0.89</v>
       </c>
       <c r="E31" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F31" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G31">
         <v>8.391</v>
@@ -2587,12 +2896,24 @@
         <v>0.19</v>
       </c>
       <c r="J31" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K31">
+        <v>-93.9</v>
+      </c>
+      <c r="L31">
+        <v>52.8</v>
+      </c>
+      <c r="M31">
+        <v>244.158</v>
+      </c>
+      <c r="N31">
+        <v>-8.165</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14">
       <c r="A32" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B32">
         <v>0.49</v>
@@ -2604,10 +2925,10 @@
         <v>0.08</v>
       </c>
       <c r="E32" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F32" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G32">
         <v>0.51</v>
@@ -2619,12 +2940,24 @@
         <v>0.00426</v>
       </c>
       <c r="J32" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K32" s="1">
+        <v>-13.06</v>
+      </c>
+      <c r="L32">
+        <v>13.3</v>
+      </c>
+      <c r="M32">
+        <v>233.76</v>
+      </c>
+      <c r="N32">
+        <v>-0.341</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14">
       <c r="A33" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B33">
         <v>2.31</v>
@@ -2636,10 +2969,10 @@
         <v>0.04</v>
       </c>
       <c r="E33" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F33" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G33">
         <v>1.292</v>
@@ -2651,12 +2984,24 @@
         <v>12.2</v>
       </c>
       <c r="J33" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K33">
+        <v>24.02</v>
+      </c>
+      <c r="L33">
+        <v>-44</v>
+      </c>
+      <c r="M33">
+        <v>139.998</v>
+      </c>
+      <c r="N33">
+        <v>31.618</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14">
       <c r="A34" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B34">
         <v>0.51</v>
@@ -2668,10 +3013,10 @@
         <v>0.04</v>
       </c>
       <c r="E34" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F34" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G34">
         <v>1.238</v>
@@ -2683,12 +3028,24 @@
         <v>0.932</v>
       </c>
       <c r="J34" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K34">
+        <v>21.64</v>
+      </c>
+      <c r="L34">
+        <v>-39.44</v>
+      </c>
+      <c r="M34">
+        <v>235.89</v>
+      </c>
+      <c r="N34">
+        <v>12.595</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14">
       <c r="A35" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B35">
         <v>2.01</v>
@@ -2700,10 +3057,10 @@
         <v>0.009</v>
       </c>
       <c r="E35" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F35" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G35">
         <v>0.531</v>
@@ -2715,12 +3072,24 @@
         <v>0.492</v>
       </c>
       <c r="J35" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K35">
+        <v>63</v>
+      </c>
+      <c r="L35">
+        <v>-96.75</v>
+      </c>
+      <c r="M35">
+        <v>196.964</v>
+      </c>
+      <c r="N35">
+        <v>31.743</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14">
       <c r="A36" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B36">
         <v>3.5</v>
@@ -2732,10 +3101,10 @@
         <v>0.2</v>
       </c>
       <c r="E36" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F36" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="G36">
         <v>0.089</v>
@@ -2747,12 +3116,12 @@
         <v>0.00113</v>
       </c>
       <c r="J36" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14">
       <c r="A37" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B37">
         <v>1.63</v>
@@ -2764,10 +3133,10 @@
         <v>0.15</v>
       </c>
       <c r="E37" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F37" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="G37">
         <v>1.274</v>
@@ -2779,12 +3148,24 @@
         <v>0.297</v>
       </c>
       <c r="J37" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K37">
+        <v>2</v>
+      </c>
+      <c r="L37">
+        <v>51</v>
+      </c>
+      <c r="M37">
+        <v>219.721</v>
+      </c>
+      <c r="N37">
+        <v>26.272</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14">
       <c r="A38" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B38">
         <v>0.83</v>
@@ -2796,10 +3177,10 @@
         <v>0.13</v>
       </c>
       <c r="E38" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F38" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="G38">
         <v>0.431</v>
@@ -2811,12 +3192,24 @@
         <v>0.0497</v>
       </c>
       <c r="J38" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K38">
+        <v>18.8</v>
+      </c>
+      <c r="L38">
+        <v>86.4</v>
+      </c>
+      <c r="M38">
+        <v>225.42</v>
+      </c>
+      <c r="N38">
+        <v>36.392</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14">
       <c r="A39" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B39">
         <v>3.82</v>
@@ -2828,10 +3221,10 @@
         <v>0.07</v>
       </c>
       <c r="E39" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F39" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G39">
         <v>0.253</v>
@@ -2843,12 +3236,24 @@
         <v>1.74</v>
       </c>
       <c r="J39" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K39">
+        <v>-2.09</v>
+      </c>
+      <c r="L39">
+        <v>29.46</v>
+      </c>
+      <c r="M39">
+        <v>228.908</v>
+      </c>
+      <c r="N39">
+        <v>43.697</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14">
       <c r="A40" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B40">
         <v>0.935</v>
@@ -2860,10 +3265,10 @@
         <v>0.055</v>
       </c>
       <c r="E40" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F40" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G40">
         <v>0.005</v>
@@ -2875,12 +3280,12 @@
         <v>441</v>
       </c>
       <c r="J40" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14">
       <c r="A41" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B41">
         <v>2.687</v>
@@ -2892,10 +3297,10 @@
         <v>0.016</v>
       </c>
       <c r="E41" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F41" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G41">
         <v>1.188</v>
@@ -2907,12 +3312,24 @@
         <v>0.504</v>
       </c>
       <c r="J41" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K41">
+        <v>-73.77</v>
+      </c>
+      <c r="L41">
+        <v>366.58</v>
+      </c>
+      <c r="M41">
+        <v>241.895</v>
+      </c>
+      <c r="N41">
+        <v>69.196</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14">
       <c r="A42" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B42">
         <v>1.16</v>
@@ -2924,10 +3341,10 @@
         <v>0.08</v>
       </c>
       <c r="E42" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F42" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G42">
         <v>1.382</v>
@@ -2939,12 +3356,24 @@
         <v>2.28</v>
       </c>
       <c r="J42" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K42">
+        <v>-104.5</v>
+      </c>
+      <c r="L42">
+        <v>49.4</v>
+      </c>
+      <c r="M42">
+        <v>252.45</v>
+      </c>
+      <c r="N42">
+        <v>86.541</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14">
       <c r="A43" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B43">
         <v>0.14</v>
@@ -2956,10 +3385,10 @@
         <v>0.09</v>
       </c>
       <c r="E43" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F43" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G43">
         <v>0.617</v>
@@ -2971,12 +3400,12 @@
         <v>2.7</v>
       </c>
       <c r="J43" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14">
       <c r="A44" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B44">
         <v>0.97</v>
@@ -2988,10 +3417,10 @@
         <v>0.14</v>
       </c>
       <c r="E44" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F44" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G44">
         <v>0.67</v>
@@ -3003,12 +3432,24 @@
         <v>1.87</v>
       </c>
       <c r="J44" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K44">
+        <v>-52.66</v>
+      </c>
+      <c r="L44">
+        <v>32.45</v>
+      </c>
+      <c r="M44">
+        <v>121.887</v>
+      </c>
+      <c r="N44">
+        <v>33.672</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14">
       <c r="A45" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B45">
         <v>2.2</v>
@@ -3020,10 +3461,10 @@
         <v>0.3</v>
       </c>
       <c r="E45" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F45" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="G45">
         <v>0.263</v>
@@ -3035,12 +3476,24 @@
         <v>4.22</v>
       </c>
       <c r="J45" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K45">
+        <v>-39.5</v>
+      </c>
+      <c r="L45">
+        <v>-12.3</v>
+      </c>
+      <c r="M45">
+        <v>313.868</v>
+      </c>
+      <c r="N45">
+        <v>-8.543</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14">
       <c r="A46" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B46">
         <v>0.47</v>
@@ -3052,10 +3505,10 @@
         <v>0.03</v>
       </c>
       <c r="E46" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F46" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G46">
         <v>0.74</v>
@@ -3067,12 +3520,24 @@
         <v>0.234</v>
       </c>
       <c r="J46" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K46">
+        <v>-73.64</v>
+      </c>
+      <c r="L46">
+        <v>-62.65</v>
+      </c>
+      <c r="M46">
+        <v>91.325</v>
+      </c>
+      <c r="N46">
+        <v>52.287</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14">
       <c r="A47" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B47">
         <v>0.62</v>
@@ -3084,10 +3549,10 @@
         <v>0.1</v>
       </c>
       <c r="E47" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F47" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G47">
         <v>1.125</v>
@@ -3099,12 +3564,24 @@
         <v>2.29</v>
       </c>
       <c r="J47" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K47">
+        <v>1.5</v>
+      </c>
+      <c r="L47">
+        <v>18.93</v>
+      </c>
+      <c r="M47">
+        <v>43.481</v>
+      </c>
+      <c r="N47">
+        <v>54.495</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14">
       <c r="A48" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B48">
         <v>0.13</v>
@@ -3116,10 +3593,10 @@
         <v>0.02</v>
       </c>
       <c r="E48" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F48" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G48">
         <v>0.748</v>
@@ -3131,12 +3608,24 @@
         <v>2.73</v>
       </c>
       <c r="J48" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K48">
+        <v>-7.61</v>
+      </c>
+      <c r="L48">
+        <v>-2.87</v>
+      </c>
+      <c r="M48">
+        <v>17.811</v>
+      </c>
+      <c r="N48">
+        <v>45.775</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14">
       <c r="A49" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B49">
         <v>0.322</v>
@@ -3148,10 +3637,10 @@
         <v>0.045</v>
       </c>
       <c r="E49" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F49" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G49">
         <v>0.709</v>
@@ -3163,12 +3652,24 @@
         <v>1.29</v>
       </c>
       <c r="J49" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K49">
+        <v>-16.79</v>
+      </c>
+      <c r="L49">
+        <v>-0.3</v>
+      </c>
+      <c r="M49">
+        <v>0.566</v>
+      </c>
+      <c r="N49">
+        <v>36.608</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14">
       <c r="A50" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B50">
         <v>0.384</v>
@@ -3180,10 +3681,10 @@
         <v>0.081</v>
       </c>
       <c r="E50" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F50" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G50">
         <v>0.257</v>
@@ -3195,12 +3696,24 @@
         <v>0.399</v>
       </c>
       <c r="J50" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K50">
+        <v>1.52</v>
+      </c>
+      <c r="L50">
+        <v>13.15</v>
+      </c>
+      <c r="M50">
+        <v>334.54</v>
+      </c>
+      <c r="N50">
+        <v>6.367</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14">
       <c r="A51" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B51">
         <v>0.91</v>
@@ -3212,10 +3725,10 @@
         <v>0.046</v>
       </c>
       <c r="E51" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F51" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G51">
         <v>0.422</v>
@@ -3227,12 +3740,24 @@
         <v>2.18</v>
       </c>
       <c r="J51" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K51">
+        <v>-26.47</v>
+      </c>
+      <c r="L51">
+        <v>-27.5</v>
+      </c>
+      <c r="M51">
+        <v>10.715</v>
+      </c>
+      <c r="N51">
+        <v>35.466</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14">
       <c r="A52" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B52">
         <v>0.59</v>
@@ -3244,10 +3769,10 @@
         <v>0.1</v>
       </c>
       <c r="E52" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F52" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G52">
         <v>1.276</v>
@@ -3259,12 +3784,24 @@
         <v>0.784</v>
       </c>
       <c r="J52" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K52">
+        <v>-10.76</v>
+      </c>
+      <c r="L52">
+        <v>23.56</v>
+      </c>
+      <c r="M52">
+        <v>5.297</v>
+      </c>
+      <c r="N52">
+        <v>27.178</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14">
       <c r="A53" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B53">
         <v>0.252</v>
@@ -3276,10 +3813,10 @@
         <v>0.019</v>
       </c>
       <c r="E53" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F53" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G53">
         <v>0.388</v>
@@ -3291,12 +3828,24 @@
         <v>0.346</v>
       </c>
       <c r="J53" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K53">
+        <v>-1.03</v>
+      </c>
+      <c r="L53">
+        <v>20.5</v>
+      </c>
+      <c r="M53">
+        <v>14.114</v>
+      </c>
+      <c r="N53">
+        <v>26.062</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14">
       <c r="A54" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B54">
         <v>0.35</v>
@@ -3308,10 +3857,10 @@
         <v>0.05</v>
       </c>
       <c r="E54" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F54" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G54">
         <v>0.804</v>
@@ -3323,12 +3872,24 @@
         <v>0.736</v>
       </c>
       <c r="J54" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K54">
+        <v>-0.73</v>
+      </c>
+      <c r="L54">
+        <v>16.92</v>
+      </c>
+      <c r="M54">
+        <v>3.229</v>
+      </c>
+      <c r="N54">
+        <v>13.561</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14">
       <c r="A55" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B55">
         <v>0</v>
@@ -3340,10 +3901,10 @@
         <v>0.2</v>
       </c>
       <c r="E55" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F55" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G55">
         <v>0.003</v>
@@ -3355,12 +3916,12 @@
         <v>1000</v>
       </c>
       <c r="J55" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14">
       <c r="A56" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B56">
         <v>2</v>
@@ -3372,10 +3933,10 @@
         <v>0.1</v>
       </c>
       <c r="E56" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F56" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G56">
         <v>0.008</v>
@@ -3387,12 +3948,12 @@
         <v>638</v>
       </c>
       <c r="J56" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14">
       <c r="A57" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B57">
         <v>0.15</v>
@@ -3404,10 +3965,10 @@
         <v>0.04</v>
       </c>
       <c r="E57" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F57" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G57">
         <v>0.419</v>
@@ -3419,12 +3980,24 @@
         <v>0.547</v>
       </c>
       <c r="J57" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K57">
+        <v>0.82</v>
+      </c>
+      <c r="L57">
+        <v>20.63</v>
+      </c>
+      <c r="M57">
+        <v>17.271</v>
+      </c>
+      <c r="N57">
+        <v>13.284</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14">
       <c r="A58" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B58">
         <v>0.28</v>
@@ -3436,10 +4009,10 @@
         <v>0.06</v>
       </c>
       <c r="E58" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F58" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G58">
         <v>2.043</v>
@@ -3451,12 +4024,24 @@
         <v>1.42</v>
       </c>
       <c r="J58" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K58">
+        <v>0.41</v>
+      </c>
+      <c r="L58">
+        <v>6.9</v>
+      </c>
+      <c r="M58">
+        <v>16.955</v>
+      </c>
+      <c r="N58">
+        <v>11.304</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14">
       <c r="A59" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B59">
         <v>2.4</v>
@@ -3468,10 +4053,10 @@
         <v>0.1</v>
       </c>
       <c r="E59" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F59" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="G59">
         <v>0.004</v>
@@ -3483,12 +4068,12 @@
         <v>723</v>
       </c>
       <c r="J59" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14">
       <c r="A60" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B60">
         <v>0.16</v>
@@ -3500,10 +4085,10 @@
         <v>0.022</v>
       </c>
       <c r="E60" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F60" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G60">
         <v>2.391</v>
@@ -3515,12 +4100,24 @@
         <v>2.42</v>
       </c>
       <c r="J60" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K60">
+        <v>-3.95</v>
+      </c>
+      <c r="L60">
+        <v>1.11</v>
+      </c>
+      <c r="M60">
+        <v>79.608</v>
+      </c>
+      <c r="N60">
+        <v>29.628</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14">
       <c r="A61" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B61">
         <v>0.4</v>
@@ -3532,10 +4129,10 @@
         <v>0.05</v>
       </c>
       <c r="E61" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F61" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="G61">
         <v>5.541</v>
@@ -3547,12 +4144,12 @@
         <v>0.0031</v>
       </c>
       <c r="J61" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14">
       <c r="A62" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B62">
         <v>0.12</v>
@@ -3564,10 +4161,10 @@
         <v>0.02</v>
       </c>
       <c r="E62" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F62" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="G62">
         <v>1.363</v>
@@ -3579,12 +4176,24 @@
         <v>5.16e-5</v>
       </c>
       <c r="J62" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K62">
+        <v>-3.572</v>
+      </c>
+      <c r="L62">
+        <v>-7.724</v>
+      </c>
+      <c r="M62">
+        <v>14.815</v>
+      </c>
+      <c r="N62">
+        <v>-0.138</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14">
       <c r="A63" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B63">
         <v>0.35</v>
@@ -3596,10 +4205,10 @@
         <v>0.06</v>
       </c>
       <c r="E63" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F63" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G63">
         <v>0.598</v>
@@ -3611,12 +4220,24 @@
         <v>0.15</v>
       </c>
       <c r="J63" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K63">
+        <v>-7.31</v>
+      </c>
+      <c r="L63">
+        <v>15.89</v>
+      </c>
+      <c r="M63">
+        <v>25.457</v>
+      </c>
+      <c r="N63">
+        <v>4.733</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14">
       <c r="A64" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B64">
         <v>0.4</v>
@@ -3628,10 +4249,10 @@
         <v>0.5</v>
       </c>
       <c r="E64" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F64" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G64">
         <v>0.003</v>
@@ -3643,12 +4264,12 @@
         <v>2.99</v>
       </c>
       <c r="J64" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="65" spans="1:14">
       <c r="A65" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B65">
         <v>0.41</v>
@@ -3660,10 +4281,10 @@
         <v>0.07</v>
       </c>
       <c r="E65" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F65" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G65">
         <v>0.687</v>
@@ -3675,12 +4296,24 @@
         <v>0.0262</v>
       </c>
       <c r="J65" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K65">
+        <v>-17.34</v>
+      </c>
+      <c r="L65">
+        <v>15</v>
+      </c>
+      <c r="M65">
+        <v>27.657</v>
+      </c>
+      <c r="N65">
+        <v>2.272</v>
+      </c>
+    </row>
+    <row r="66" spans="1:14">
       <c r="A66" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B66">
         <v>0.657</v>
@@ -3692,10 +4325,10 @@
         <v>0.008</v>
       </c>
       <c r="E66" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F66" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G66">
         <v>1.653</v>
@@ -3707,12 +4340,24 @@
         <v>1.75</v>
       </c>
       <c r="J66" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K66">
+        <v>-31.21</v>
+      </c>
+      <c r="L66">
+        <v>-29.1</v>
+      </c>
+      <c r="M66">
+        <v>86.078</v>
+      </c>
+      <c r="N66">
+        <v>23.819</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14">
       <c r="A67" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B67">
         <v>6.2</v>
@@ -3724,10 +4369,10 @@
         <v>0.6</v>
       </c>
       <c r="E67" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="F67" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="G67">
         <v>7.055</v>
@@ -3739,12 +4384,24 @@
         <v>0.376</v>
       </c>
       <c r="J67" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="68" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K67">
+        <v>325.9</v>
+      </c>
+      <c r="L67">
+        <v>-59.22</v>
+      </c>
+      <c r="M67">
+        <v>358.599</v>
+      </c>
+      <c r="N67">
+        <v>-17.215</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14">
       <c r="A68" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B68">
         <v>0.5</v>
@@ -3756,10 +4413,10 @@
         <v>0.6</v>
       </c>
       <c r="E68" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F68" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="G68">
         <v>0.612</v>
@@ -3771,12 +4428,12 @@
         <v>4.66</v>
       </c>
       <c r="J68" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="69" spans="1:10">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14">
       <c r="A69" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B69">
         <v>0.51</v>
@@ -3788,10 +4445,10 @@
         <v>0.04</v>
       </c>
       <c r="E69" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F69" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G69">
         <v>1.782</v>
@@ -3803,12 +4460,24 @@
         <v>1.72</v>
       </c>
       <c r="J69" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="70" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K69">
+        <v>-7.54</v>
+      </c>
+      <c r="L69">
+        <v>-18.2</v>
+      </c>
+      <c r="M69">
+        <v>25.979</v>
+      </c>
+      <c r="N69">
+        <v>-6.441</v>
+      </c>
+    </row>
+    <row r="70" spans="1:14">
       <c r="A70" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B70">
         <v>0.024</v>
@@ -3820,10 +4489,10 @@
         <v>0.022</v>
       </c>
       <c r="E70" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F70" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G70">
         <v>2.233</v>
@@ -3835,12 +4504,12 @@
         <v>0.348</v>
       </c>
       <c r="J70" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="71" spans="1:10">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="71" spans="1:14">
       <c r="A71" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B71">
         <v>0.185</v>
@@ -3852,10 +4521,10 @@
         <v>0.023</v>
       </c>
       <c r="E71" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F71" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G71">
         <v>0.521</v>
@@ -3867,12 +4536,24 @@
         <v>1.03</v>
       </c>
       <c r="J71" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="72" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K71">
+        <v>-5.28</v>
+      </c>
+      <c r="L71">
+        <v>-8.94</v>
+      </c>
+      <c r="M71">
+        <v>47.881</v>
+      </c>
+      <c r="N71">
+        <v>1.592</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14">
       <c r="A72" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B72">
         <v>0.142</v>
@@ -3884,10 +4565,10 @@
         <v>0.007</v>
       </c>
       <c r="E72" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F72" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G72">
         <v>0.195</v>
@@ -3899,12 +4580,24 @@
         <v>0.0429</v>
       </c>
       <c r="J72" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="73" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K72">
+        <v>-1.28</v>
+      </c>
+      <c r="L72">
+        <v>3.81</v>
+      </c>
+      <c r="M72">
+        <v>48.26</v>
+      </c>
+      <c r="N72">
+        <v>0.624</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14">
       <c r="A73" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B73">
         <v>0.16</v>
@@ -3916,10 +4609,10 @@
         <v>0.04</v>
       </c>
       <c r="E73" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F73" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G73">
         <v>1.272</v>
@@ -3931,12 +4624,24 @@
         <v>0.263</v>
       </c>
       <c r="J73" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="74" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K73">
+        <v>10.11</v>
+      </c>
+      <c r="L73">
+        <v>-4.7</v>
+      </c>
+      <c r="M73">
+        <v>36.506</v>
+      </c>
+      <c r="N73">
+        <v>-6.151</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14">
       <c r="A74" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B74">
         <v>2.77</v>
@@ -3948,10 +4653,10 @@
         <v>0.07</v>
       </c>
       <c r="E74" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F74" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="G74">
         <v>0.227</v>
@@ -3963,12 +4668,24 @@
         <v>0.31</v>
       </c>
       <c r="J74" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="75" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K74">
+        <v>94.09</v>
+      </c>
+      <c r="L74">
+        <v>42.99</v>
+      </c>
+      <c r="M74">
+        <v>47.382</v>
+      </c>
+      <c r="N74">
+        <v>-3.885</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14">
       <c r="A75" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B75">
         <v>0.22</v>
@@ -3980,10 +4697,10 @@
         <v>0.12</v>
       </c>
       <c r="E75" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F75" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G75">
         <v>0.359</v>
@@ -3995,12 +4712,12 @@
         <v>0.0947</v>
       </c>
       <c r="J75" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="76" spans="1:10">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14">
       <c r="A76" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B76">
         <v>0.318</v>
@@ -4012,10 +4729,10 @@
         <v>0.029</v>
       </c>
       <c r="E76" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F76" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G76">
         <v>0.201</v>
@@ -4027,12 +4744,24 @@
         <v>0.495</v>
       </c>
       <c r="J76" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="77" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K76">
+        <v>-10.04</v>
+      </c>
+      <c r="L76">
+        <v>-13.06</v>
+      </c>
+      <c r="M76">
+        <v>60.836</v>
+      </c>
+      <c r="N76">
+        <v>2.27</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14">
       <c r="A77" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B77">
         <v>0.35</v>
@@ -4044,10 +4773,10 @@
         <v>0.03</v>
       </c>
       <c r="E77" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F77" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G77">
         <v>0.002</v>
@@ -4059,12 +4788,12 @@
         <v>23.5</v>
       </c>
       <c r="J77" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="78" spans="1:10">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="78" spans="1:14">
       <c r="A78" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B78">
         <v>0.424</v>
@@ -4076,10 +4805,10 @@
         <v>0.01</v>
       </c>
       <c r="E78" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F78" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G78">
         <v>0.581</v>
@@ -4091,12 +4820,24 @@
         <v>20.2</v>
       </c>
       <c r="J78" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="79" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K78">
+        <v>-6.19</v>
+      </c>
+      <c r="L78">
+        <v>-10.59</v>
+      </c>
+      <c r="M78">
+        <v>34.101</v>
+      </c>
+      <c r="N78">
+        <v>-20.304</v>
+      </c>
+    </row>
+    <row r="79" spans="1:14">
       <c r="A79" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B79">
         <v>0.48</v>
@@ -4108,10 +4849,10 @@
         <v>0.12</v>
       </c>
       <c r="E79" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F79" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G79">
         <v>0.005</v>
@@ -4123,12 +4864,12 @@
         <v>1720</v>
       </c>
       <c r="J79" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="80" spans="1:10">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="80" spans="1:14">
       <c r="A80" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B80">
         <v>1.03</v>
@@ -4140,10 +4881,10 @@
         <v>0.1</v>
       </c>
       <c r="E80" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F80" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G80">
         <v>0.558</v>
@@ -4155,12 +4896,24 @@
         <v>5.97</v>
       </c>
       <c r="J80" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="81" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K80">
+        <v>-2.6</v>
+      </c>
+      <c r="L80">
+        <v>-6.2</v>
+      </c>
+      <c r="M80">
+        <v>68.099</v>
+      </c>
+      <c r="N80">
+        <v>-3.983</v>
+      </c>
+    </row>
+    <row r="81" spans="1:14">
       <c r="A81" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B81">
         <v>0.37</v>
@@ -4172,10 +4925,10 @@
         <v>0.12</v>
       </c>
       <c r="E81" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F81" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G81">
         <v>0.343</v>
@@ -4187,12 +4940,24 @@
         <v>0.287</v>
       </c>
       <c r="J81" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="82" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K81">
+        <v>-4.4</v>
+      </c>
+      <c r="L81">
+        <v>-23.6</v>
+      </c>
+      <c r="M81">
+        <v>68.863</v>
+      </c>
+      <c r="N81">
+        <v>-4.671</v>
+      </c>
+    </row>
+    <row r="82" spans="1:14">
       <c r="A82" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B82">
         <v>0.5</v>
@@ -4204,10 +4969,10 @@
         <v>0.07</v>
       </c>
       <c r="E82" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F82" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="G82">
         <v>0.529</v>
@@ -4219,12 +4984,24 @@
         <v>0.274</v>
       </c>
       <c r="J82" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="83" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K82">
+        <v>-5.23</v>
+      </c>
+      <c r="L82">
+        <v>11.5</v>
+      </c>
+      <c r="M82">
+        <v>87.862</v>
+      </c>
+      <c r="N82">
+        <v>8.38</v>
+      </c>
+    </row>
+    <row r="83" spans="1:14">
       <c r="A83" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="B83">
         <v>0.31</v>
@@ -4236,10 +5013,10 @@
         <v>0.08</v>
       </c>
       <c r="E83" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F83" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G83">
         <v>1.138</v>
@@ -4251,12 +5028,24 @@
         <v>9.88</v>
       </c>
       <c r="J83" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="84" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K83">
+        <v>-10.48</v>
+      </c>
+      <c r="L83">
+        <v>0.66</v>
+      </c>
+      <c r="M83">
+        <v>61.112</v>
+      </c>
+      <c r="N83">
+        <v>-16.838</v>
+      </c>
+    </row>
+    <row r="84" spans="1:14">
       <c r="A84" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B84">
         <v>0.167</v>
@@ -4268,10 +5057,10 @@
         <v>0.042</v>
       </c>
       <c r="E84" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F84" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G84">
         <v>1.547</v>
@@ -4283,12 +5072,24 @@
         <v>1.67</v>
       </c>
       <c r="J84" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="85" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K84">
+        <v>10.76</v>
+      </c>
+      <c r="L84">
+        <v>-4.3</v>
+      </c>
+      <c r="M84">
+        <v>42.678</v>
+      </c>
+      <c r="N84">
+        <v>-27.387</v>
+      </c>
+    </row>
+    <row r="85" spans="1:14">
       <c r="A85" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="B85">
         <v>1.38</v>
@@ -4300,10 +5101,10 @@
         <v>0.64</v>
       </c>
       <c r="E85" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F85" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="G85">
         <v>1.962</v>
@@ -4315,12 +5116,12 @@
         <v>0.283</v>
       </c>
       <c r="J85" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="86" spans="1:10">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="86" spans="1:14">
       <c r="A86" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B86">
         <v>0.17</v>
@@ -4332,10 +5133,10 @@
         <v>0.03</v>
       </c>
       <c r="E86" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F86" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G86">
         <v>0.221</v>
@@ -4347,12 +5148,24 @@
         <v>0.951</v>
       </c>
       <c r="J86" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="87" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K86">
+        <v>1.04</v>
+      </c>
+      <c r="L86">
+        <v>-2.46</v>
+      </c>
+      <c r="M86">
+        <v>79.133</v>
+      </c>
+      <c r="N86">
+        <v>-5.589</v>
+      </c>
+    </row>
+    <row r="87" spans="1:14">
       <c r="A87" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B87">
         <v>0.704</v>
@@ -4364,10 +5177,10 @@
         <v>0.022</v>
       </c>
       <c r="E87" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F87" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G87">
         <v>1.203</v>
@@ -4379,12 +5192,24 @@
         <v>0.727</v>
       </c>
       <c r="J87" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="88" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K87">
+        <v>-27.96</v>
+      </c>
+      <c r="L87">
+        <v>-54.46</v>
+      </c>
+      <c r="M87">
+        <v>74.993</v>
+      </c>
+      <c r="N87">
+        <v>-14.025</v>
+      </c>
+    </row>
+    <row r="88" spans="1:14">
       <c r="A88" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B88">
         <v>0.45</v>
@@ -4396,10 +5221,10 @@
         <v>0.07</v>
       </c>
       <c r="E88" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F88" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G88">
         <v>1.015</v>
@@ -4411,12 +5236,24 @@
         <v>2.25</v>
       </c>
       <c r="J88" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="89" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K88">
+        <v>9.5</v>
+      </c>
+      <c r="L88">
+        <v>8.84</v>
+      </c>
+      <c r="M88">
+        <v>89.003</v>
+      </c>
+      <c r="N88">
+        <v>-1.266</v>
+      </c>
+    </row>
+    <row r="89" spans="1:14">
       <c r="A89" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B89">
         <v>3.1</v>
@@ -4428,10 +5265,10 @@
         <v>0.55</v>
       </c>
       <c r="E89" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F89" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="G89">
         <v>0.005</v>
@@ -4443,12 +5280,12 @@
         <v>380</v>
       </c>
       <c r="J89" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="90" spans="1:10">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="90" spans="1:14">
       <c r="A90" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B90">
         <v>6.05</v>
@@ -4460,10 +5297,10 @@
         <v>0.56</v>
       </c>
       <c r="E90" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F90" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="G90">
         <v>8.51</v>
@@ -4475,12 +5312,24 @@
         <v>27.2</v>
       </c>
       <c r="J90" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="91" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K90">
+        <v>-57.9</v>
+      </c>
+      <c r="L90">
+        <v>-155.9</v>
+      </c>
+      <c r="M90">
+        <v>2.794</v>
+      </c>
+      <c r="N90">
+        <v>-49.466</v>
+      </c>
+    </row>
+    <row r="91" spans="1:14">
       <c r="A91" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B91">
         <v>0.36</v>
@@ -4492,10 +5341,10 @@
         <v>0.06</v>
       </c>
       <c r="E91" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F91" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G91">
         <v>0.38</v>
@@ -4507,12 +5356,24 @@
         <v>3.58</v>
       </c>
       <c r="J91" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="92" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K91">
+        <v>15.81</v>
+      </c>
+      <c r="L91">
+        <v>11.16</v>
+      </c>
+      <c r="M91">
+        <v>104.255</v>
+      </c>
+      <c r="N91">
+        <v>7.412</v>
+      </c>
+    </row>
+    <row r="92" spans="1:14">
       <c r="A92" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B92">
         <v>0.03</v>
@@ -4524,10 +5385,10 @@
         <v>0.08</v>
       </c>
       <c r="E92" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F92" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G92">
         <v>0.332</v>
@@ -4539,12 +5400,12 @@
         <v>0.0521</v>
       </c>
       <c r="J92" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="93" spans="1:10">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="93" spans="1:14">
       <c r="A93" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B93">
         <v>0.28</v>
@@ -4556,10 +5417,10 @@
         <v>0.06</v>
       </c>
       <c r="E93" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F93" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G93">
         <v>1.525</v>
@@ -4571,12 +5432,24 @@
         <v>0.704</v>
       </c>
       <c r="J93" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="94" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K93">
+        <v>16.13</v>
+      </c>
+      <c r="L93">
+        <v>4.12</v>
+      </c>
+      <c r="M93">
+        <v>90.488</v>
+      </c>
+      <c r="N93">
+        <v>-11.341</v>
+      </c>
+    </row>
+    <row r="94" spans="1:14">
       <c r="A94" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B94">
         <v>0.27</v>
@@ -4588,10 +5461,10 @@
         <v>0.12</v>
       </c>
       <c r="E94" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F94" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G94">
         <v>1.005</v>
@@ -4603,12 +5476,12 @@
         <v>3.21</v>
       </c>
       <c r="J94" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="95" spans="1:10">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="95" spans="1:14">
       <c r="A95" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B95">
         <v>1.2</v>
@@ -4620,10 +5493,10 @@
         <v>0.2</v>
       </c>
       <c r="E95" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F95" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G95">
         <v>0.683</v>
@@ -4635,12 +5508,24 @@
         <v>0.112</v>
       </c>
       <c r="J95" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="96" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K95">
+        <v>147.2</v>
+      </c>
+      <c r="L95">
+        <v>126.5</v>
+      </c>
+      <c r="M95">
+        <v>108.638</v>
+      </c>
+      <c r="N95">
+        <v>6.846</v>
+      </c>
+    </row>
+    <row r="96" spans="1:14">
       <c r="A96" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B96">
         <v>0.26</v>
@@ -4652,10 +5537,10 @@
         <v>0.07</v>
       </c>
       <c r="E96" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F96" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="G96">
         <v>0.477</v>
@@ -4667,12 +5552,24 @@
         <v>1.15</v>
       </c>
       <c r="J96" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="97" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K96">
+        <v>-10.5</v>
+      </c>
+      <c r="L96">
+        <v>-17.49</v>
+      </c>
+      <c r="M96">
+        <v>69.256</v>
+      </c>
+      <c r="N96">
+        <v>-50.62</v>
+      </c>
+    </row>
+    <row r="97" spans="1:14">
       <c r="A97" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B97">
         <v>0.223</v>
@@ -4684,10 +5581,10 @@
         <v>0.028</v>
       </c>
       <c r="E97" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F97" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G97">
         <v>1.576</v>
@@ -4699,12 +5596,24 @@
         <v>0.863</v>
       </c>
       <c r="J97" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="98" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K97">
+        <v>-3.7</v>
+      </c>
+      <c r="L97">
+        <v>-15.63</v>
+      </c>
+      <c r="M97">
+        <v>97.721</v>
+      </c>
+      <c r="N97">
+        <v>-26.657</v>
+      </c>
+    </row>
+    <row r="98" spans="1:14">
       <c r="A98" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B98">
         <v>0.93</v>
@@ -4716,10 +5625,10 @@
         <v>0.07</v>
       </c>
       <c r="E98" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F98" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G98">
         <v>0.349</v>
@@ -4731,12 +5640,24 @@
         <v>4.93</v>
       </c>
       <c r="J98" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="99" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K98">
+        <v>24.15</v>
+      </c>
+      <c r="L98">
+        <v>5.95</v>
+      </c>
+      <c r="M98">
+        <v>104.41</v>
+      </c>
+      <c r="N98">
+        <v>-16.422</v>
+      </c>
+    </row>
+    <row r="99" spans="1:14">
       <c r="A99" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B99">
         <v>0.51</v>
@@ -4748,10 +5669,10 @@
         <v>0.05</v>
       </c>
       <c r="E99" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F99" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G99">
         <v>1.445</v>
@@ -4763,12 +5684,24 @@
         <v>2.19</v>
       </c>
       <c r="J99" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="100" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K99">
+        <v>8.49</v>
+      </c>
+      <c r="L99">
+        <v>0.19</v>
+      </c>
+      <c r="M99">
+        <v>95.831</v>
+      </c>
+      <c r="N99">
+        <v>-36.075</v>
+      </c>
+    </row>
+    <row r="100" spans="1:14">
       <c r="A100" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B100">
         <v>0.275</v>
@@ -4780,10 +5713,10 @@
         <v>0.036</v>
       </c>
       <c r="E100" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F100" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G100">
         <v>1.181</v>
@@ -4795,12 +5728,24 @@
         <v>1.37</v>
       </c>
       <c r="J100" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="101" spans="1:10">
+        <v>17</v>
+      </c>
+      <c r="K100">
+        <v>37.38</v>
+      </c>
+      <c r="L100">
+        <v>-20.21</v>
+      </c>
+      <c r="M100">
+        <v>83.798</v>
+      </c>
+      <c r="N100">
+        <v>-64.015</v>
+      </c>
+    </row>
+    <row r="101" spans="1:14">
       <c r="A101" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B101">
         <v>0.41</v>
@@ -4812,10 +5757,10 @@
         <v>0.04</v>
       </c>
       <c r="E101" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="F101" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="G101">
         <v>0.945</v>
@@ -4827,7 +5772,19 @@
         <v>0.092</v>
       </c>
       <c r="J101" t="s">
-        <v>13</v>
+        <v>17</v>
+      </c>
+      <c r="K101">
+        <v>22.76</v>
+      </c>
+      <c r="L101">
+        <v>4.9</v>
+      </c>
+      <c r="M101">
+        <v>116.239</v>
+      </c>
+      <c r="N101">
+        <v>-0.194</v>
       </c>
     </row>
   </sheetData>

</xml_diff>